<commit_message>
Fixing all old test files with wrong cell A1
</commit_message>
<xml_diff>
--- a/test-files/adjacency-matrix-modifications/data-types/data-type-header-accounting-input.xlsx
+++ b/test-files/adjacency-matrix-modifications/data-types/data-type-header-accounting-input.xlsx
@@ -1,11 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27430"/>
-  <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14240" firstSheet="7" activeTab="8"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook" autoCompressPictures="false" showInkAnnotation="false"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
@@ -18,194 +14,46 @@
     <sheet name="network" sheetId="9" r:id="rId9"/>
     <sheet name="network_weights" sheetId="10" r:id="rId10"/>
     <sheet name="network_optimized_b" sheetId="11" r:id="rId11"/>
-    <sheet name="concentration_sigmas" sheetId="13" r:id="rId12"/>
+    <sheet name="concentration_sigmas" sheetId="12" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="125725" concurrentCalc="0"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="49">
-  <si>
-    <t>SystematicName</t>
-  </si>
-  <si>
-    <t>StandardName</t>
-  </si>
-  <si>
-    <t>YKL112W</t>
-  </si>
-  <si>
-    <t>ABF1</t>
-  </si>
-  <si>
-    <t>YLR131C</t>
-  </si>
-  <si>
-    <t>ACE2</t>
-  </si>
-  <si>
-    <t>YGL071W</t>
-  </si>
-  <si>
-    <t>AFT1</t>
-  </si>
-  <si>
-    <t>YOR028C</t>
-  </si>
-  <si>
-    <t>CIN5</t>
-  </si>
-  <si>
-    <t>YPL177C</t>
-  </si>
-  <si>
-    <t>CUP9</t>
-  </si>
-  <si>
-    <t>YPR104C</t>
-  </si>
-  <si>
-    <t>FHL1</t>
-  </si>
-  <si>
-    <t>YGL181W</t>
-  </si>
-  <si>
-    <t>GTS1</t>
-  </si>
-  <si>
-    <t>YOL089C</t>
-  </si>
-  <si>
-    <t>HAL9</t>
-  </si>
-  <si>
-    <t>YGL073W</t>
-  </si>
-  <si>
-    <t>HSF1</t>
-  </si>
-  <si>
-    <t>YMR021C</t>
-  </si>
-  <si>
-    <t>MAC1</t>
-  </si>
-  <si>
-    <t>YOL116W</t>
-  </si>
-  <si>
-    <t>MSN1</t>
-  </si>
-  <si>
-    <t>YKL062W</t>
-  </si>
-  <si>
-    <t>MSN4</t>
-  </si>
-  <si>
-    <t>YDR043C</t>
-  </si>
-  <si>
-    <t>NRG1</t>
-  </si>
-  <si>
-    <t>YKL043W</t>
-  </si>
-  <si>
-    <t>PHD1</t>
-  </si>
-  <si>
-    <t>YNL216W</t>
-  </si>
-  <si>
-    <t>RAP1</t>
-  </si>
-  <si>
-    <t>YBR049C</t>
-  </si>
-  <si>
-    <t>REB1</t>
-  </si>
-  <si>
-    <t>YPR065W</t>
-  </si>
-  <si>
-    <t>ROX1</t>
-  </si>
-  <si>
-    <t>YER169W</t>
-  </si>
-  <si>
-    <t>RPH1</t>
-  </si>
-  <si>
-    <t>YHR206W</t>
-  </si>
-  <si>
-    <t>SKN7</t>
-  </si>
-  <si>
-    <t>YML007W</t>
-  </si>
-  <si>
-    <t>YAP1</t>
-  </si>
-  <si>
-    <t>YDR259C</t>
-  </si>
-  <si>
-    <t>YAP6</t>
-  </si>
-  <si>
-    <t>DegradationRate</t>
-  </si>
-  <si>
-    <t>production_rates</t>
-  </si>
-  <si>
-    <t>time</t>
-  </si>
-  <si>
-    <t>rows genes affected/cols genes controlling</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="2">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="10"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -225,26 +73,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="5">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -569,95 +408,91 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" t="s">
-        <v>25</v>
-      </c>
-      <c r="N1" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" t="s">
-        <v>29</v>
-      </c>
-      <c r="P1" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>33</v>
-      </c>
-      <c r="R1" t="s">
-        <v>35</v>
-      </c>
-      <c r="S1" t="s">
-        <v>37</v>
-      </c>
-      <c r="T1" t="s">
-        <v>39</v>
-      </c>
-      <c r="U1" t="s">
-        <v>41</v>
-      </c>
-      <c r="V1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:22">
-      <c r="A2" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>rows genes affected/cols genes controlling</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ABF1</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ACE2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>AFT1</v>
+      </c>
+      <c r="E1" t="str">
+        <v>CIN5</v>
+      </c>
+      <c r="F1" t="str">
+        <v>CUP9</v>
+      </c>
+      <c r="G1" t="str">
+        <v>FHL1</v>
+      </c>
+      <c r="H1" t="str">
+        <v>GTS1</v>
+      </c>
+      <c r="I1" t="str">
+        <v>HAL9</v>
+      </c>
+      <c r="J1" t="str">
+        <v>HSF1</v>
+      </c>
+      <c r="K1" t="str">
+        <v>MAC1</v>
+      </c>
+      <c r="L1" t="str">
+        <v>MSN1</v>
+      </c>
+      <c r="M1" t="str">
+        <v>MSN4</v>
+      </c>
+      <c r="N1" t="str">
+        <v>NRG1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>PHD1</v>
+      </c>
+      <c r="P1" t="str">
+        <v>RAP1</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>REB1</v>
+      </c>
+      <c r="R1" t="str">
+        <v>ROX1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>RPH1</v>
+      </c>
+      <c r="T1" t="str">
+        <v>SKN7</v>
+      </c>
+      <c r="U1" t="str">
+        <v>YAP1</v>
+      </c>
+      <c r="V1" t="str">
+        <v>YAP6</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -723,9 +558,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:22">
-      <c r="A3" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -791,9 +626,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
-      <c r="A4" t="s">
-        <v>7</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -859,9 +694,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22">
-      <c r="A5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -927,9 +762,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:22">
-      <c r="A6" t="s">
-        <v>11</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -995,9 +830,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
-      <c r="A7" t="s">
-        <v>13</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1063,9 +898,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
-      <c r="A8" t="s">
-        <v>15</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1131,9 +966,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22">
-      <c r="A9" t="s">
-        <v>17</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1199,9 +1034,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22">
-      <c r="A10" t="s">
-        <v>19</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1267,9 +1102,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
-      <c r="A11" t="s">
-        <v>21</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1335,9 +1170,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
-      <c r="A12" t="s">
-        <v>23</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1403,9 +1238,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
-      <c r="A13" t="s">
-        <v>25</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1471,9 +1306,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
-      <c r="A14" t="s">
-        <v>27</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1539,9 +1374,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22">
-      <c r="A15" t="s">
-        <v>29</v>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1607,9 +1442,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
-      <c r="A16" t="s">
-        <v>31</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1675,9 +1510,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
-      <c r="A17" t="s">
-        <v>33</v>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>REB1</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1743,9 +1578,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:22">
-      <c r="A18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1811,9 +1646,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
-      <c r="A19" t="s">
-        <v>37</v>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1879,9 +1714,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:22">
-      <c r="A20" t="s">
-        <v>39</v>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1947,9 +1782,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
-      <c r="A21" t="s">
-        <v>41</v>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2015,9 +1850,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:22">
-      <c r="A22" t="s">
-        <v>43</v>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -2085,256 +1920,253 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:V22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>b</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
-        <v>0.65031415394516434</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>0.6503141539451643</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
-        <v>1.1608735890637201</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>1.16087358906372</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
         <v>4.723434337016859</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
         <v>2.2093965892822576</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
         <v>1.4838022384341765</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
-        <v>4.3880758825533226</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+        <v>4.388075882553323</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
         <v>1.4292526942022845</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
         <v>0.21204144369617425</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
-        <v>3.1826495298927981</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>3.182649529892798</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
-        <v>0.83154851292891641</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+        <v>0.8315485129289164</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
         <v>5.312232618008994</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
         <v>0.30350389708240194</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
         <v>1.090960278752473</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
-        <v>2.9644811435403602</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>2.96448114354036</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
         <v>1.411956405672939</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
         <v>1.0908187404229068</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
         <v>3.0278217120091173</v>
@@ -2342,25 +2174,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
       </c>
       <c r="C1">
         <v>15</v>
@@ -2372,236 +2201,236 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
-        <v>0.91727409105065705</v>
+        <v>0.917274091050657</v>
       </c>
       <c r="D2">
-        <v>0.44210879486447602</v>
+        <v>0.442108794864476</v>
       </c>
       <c r="E2">
-        <v>0.69315515241602899</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>0.693155152416029</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
-        <v>0.71685637353245302</v>
+        <v>0.716856373532453</v>
       </c>
       <c r="D3">
         <v>0.641384013885964</v>
       </c>
       <c r="E3">
-        <v>0.92245951116837099</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>0.922459511168371</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
-        <v>0.44470247868505602</v>
+        <v>0.444702478685056</v>
       </c>
       <c r="D4">
-        <v>0.53164120946850402</v>
+        <v>0.531641209468504</v>
       </c>
       <c r="E4">
         <v>0.320493749001932</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
-        <v>0.81727687981679498</v>
+        <v>0.817276879816795</v>
       </c>
       <c r="D5">
-        <v>0.95726655288635398</v>
+        <v>0.957266552886354</v>
       </c>
       <c r="E5">
-        <v>0.70281582595053704</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+        <v>0.702815825950537</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
-        <v>1.0967850406720701</v>
+        <v>1.09678504067207</v>
       </c>
       <c r="D6">
-        <v>0.52970920759899298</v>
+        <v>0.529709207598993</v>
       </c>
       <c r="E6">
-        <v>0.80891828959740097</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+        <v>0.808918289597401</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
-        <v>0.42580145197082703</v>
+        <v>0.425801451970827</v>
       </c>
       <c r="D7">
-        <v>0.63499396842678302</v>
+        <v>0.634993968426783</v>
       </c>
       <c r="E7">
-        <v>0.78157727034137603</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+        <v>0.781577270341376</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
         <v>0.404638632823907</v>
       </c>
       <c r="D8">
-        <v>0.58989131883839296</v>
+        <v>0.589891318838393</v>
       </c>
       <c r="E8">
-        <v>0.60748498565234699</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+        <v>0.607484985652347</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
-        <v>0.68943520086600596</v>
+        <v>0.689435200866006</v>
       </c>
       <c r="D9">
-        <v>1.8955428214225301</v>
+        <v>1.89554282142253</v>
       </c>
       <c r="E9">
-        <v>0.54723644512184799</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+        <v>0.547236445121848</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
-        <v>0.97726406268218102</v>
+        <v>0.977264062682181</v>
       </c>
       <c r="D10">
-        <v>0.72420652572711597</v>
+        <v>0.724206525727116</v>
       </c>
       <c r="E10">
         <v>1.09985790153451</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
-        <v>0.72504670083612599</v>
+        <v>0.725046700836126</v>
       </c>
       <c r="D11">
-        <v>0.20779307950352699</v>
+        <v>0.207793079503527</v>
       </c>
       <c r="E11">
-        <v>0.65825511050072905</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+        <v>0.658255110500729</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
-        <v>0.51852196117730698</v>
+        <v>0.518521961177307</v>
       </c>
       <c r="D12">
-        <v>0.88709656674279203</v>
+        <v>0.887096566742792</v>
       </c>
       <c r="E12">
         <v>0.248881921070051</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
-        <v>1.6409513470958299</v>
+        <v>1.64095134709583</v>
       </c>
       <c r="D13">
         <v>1.01226276719667</v>
       </c>
       <c r="E13">
-        <v>1.2436321609087699</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+        <v>1.24363216090877</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
-        <v>0.56438763790471502</v>
+        <v>0.564387637904715</v>
       </c>
       <c r="D14">
         <v>0.637046148638169</v>
       </c>
       <c r="E14">
-        <v>0.76246682595887705</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>0.762466825958877</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
-        <v>0.48729361226630702</v>
+        <v>0.487293612266307</v>
       </c>
       <c r="D15">
         <v>0.460208681767377</v>
@@ -2610,120 +2439,120 @@
         <v>0.389622153973187</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
         <v>1.72099674768658</v>
       </c>
       <c r="D16">
-        <v>0.85831878781873805</v>
+        <v>0.858318787818738</v>
       </c>
       <c r="E16">
-        <v>0.44772738659776701</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+        <v>0.447727386597767</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
-        <v>0.50452893050955805</v>
+        <v>0.504528930509558</v>
       </c>
       <c r="D17">
-        <v>0.75370009518917203</v>
+        <v>0.753700095189172</v>
       </c>
       <c r="E17">
         <v>1.07122097617887</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
-        <v>1.1966265259256601</v>
+        <v>1.19662652592566</v>
       </c>
       <c r="D18">
-        <v>1.1801382981458799</v>
+        <v>1.18013829814588</v>
       </c>
       <c r="E18">
-        <v>0.35000209622478101</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+        <v>0.350002096224781</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
         <v>1.48156426614991</v>
       </c>
       <c r="D19">
-        <v>1.7277862291131501</v>
+        <v>1.72778622911315</v>
       </c>
       <c r="E19">
-        <v>0.89902628670097295</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>0.899026286700973</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
         <v>1.10568541431009</v>
       </c>
       <c r="D20">
-        <v>0.84212726958299999</v>
+        <v>0.842127269583</v>
       </c>
       <c r="E20">
-        <v>0.74688657635395606</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+        <v>0.746886576353956</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
-        <v>0.65898902973629203</v>
+        <v>0.658989029736292</v>
       </c>
       <c r="D21">
-        <v>0.43418451003840802</v>
+        <v>0.434184510038408</v>
       </c>
       <c r="E21">
-        <v>0.53794081650927705</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+        <v>0.537940816509277</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
-        <v>0.40923963868872798</v>
+        <v>0.409239638688728</v>
       </c>
       <c r="D22">
-        <v>0.28048461336490499</v>
+        <v>0.280484613364905</v>
       </c>
       <c r="E22">
         <v>0.287254982132019</v>
@@ -2731,53 +2560,44 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
       </c>
       <c r="C1">
         <v>15</v>
@@ -2789,29 +2609,29 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
-        <v>-1.1802129985963199</v>
+        <v>-1.18021299859632</v>
       </c>
       <c r="D2">
         <v>-1.35534786374789</v>
       </c>
       <c r="E2">
-        <v>-2.2843447109758301</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>-2.28434471097583</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
         <v>-0.168317226797601</v>
@@ -2820,219 +2640,219 @@
         <v>0.159981381075125</v>
       </c>
       <c r="E3">
-        <v>-8.4072251269262696E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>-0.0840722512692627</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
         <v>0.110916570402342</v>
       </c>
       <c r="D4">
-        <v>0.34518552113600498</v>
+        <v>0.345185521136005</v>
       </c>
       <c r="E4">
-        <v>0.29611171632314098</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>0.296111716323141</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
-        <v>0.57398886351082801</v>
+        <v>0.573988863510828</v>
       </c>
       <c r="D5">
-        <v>0.90044244474717405</v>
+        <v>0.900442444747174</v>
       </c>
       <c r="E5">
         <v>1.75845186354745</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
-        <v>-0.34976006979129598</v>
+        <v>-0.349760069791296</v>
       </c>
       <c r="D6">
-        <v>-0.97753185452394098</v>
+        <v>-0.977531854523941</v>
       </c>
       <c r="E6">
-        <v>-0.76236366760055096</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+        <v>-0.762363667600551</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
-        <v>-4.4276309137313001E-2</v>
+        <v>-0.044276309137313</v>
       </c>
       <c r="D7">
-        <v>0.24181613073483699</v>
+        <v>0.241816130734837</v>
       </c>
       <c r="E7">
-        <v>0.62853290835895503</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+        <v>0.628532908358955</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
         <v>-0.220356822259166</v>
       </c>
       <c r="D8">
-        <v>-0.11669113002233999</v>
+        <v>-0.11669113002234</v>
       </c>
       <c r="E8">
-        <v>-8.7143718210927298E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+        <v>-0.0871437182109273</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
-        <v>-0.16064769982257401</v>
+        <v>-0.160647699822574</v>
       </c>
       <c r="D9">
-        <v>0.20886614963405101</v>
+        <v>0.208866149634051</v>
       </c>
       <c r="E9">
-        <v>0.84698244904192099</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+        <v>0.846982449041921</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
-        <v>-0.97765022692802495</v>
+        <v>-0.977650226928025</v>
       </c>
       <c r="D10">
-        <v>-1.1044654053835501</v>
+        <v>-1.10446540538355</v>
       </c>
       <c r="E10">
-        <v>-0.73218305564943398</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+        <v>-0.732183055649434</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
-        <v>0.61308674677972397</v>
+        <v>0.613086746779724</v>
       </c>
       <c r="D11">
-        <v>0.49022096483014099</v>
+        <v>0.490220964830141</v>
       </c>
       <c r="E11">
-        <v>0.45176478094112998</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+        <v>0.45176478094113</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
         <v>0.124182913442922</v>
       </c>
       <c r="D12">
-        <v>-0.42545856172641699</v>
+        <v>-0.425458561726417</v>
       </c>
       <c r="E12">
-        <v>-0.48116619434522001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+        <v>-0.48116619434522</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
-        <v>0.98300627566904297</v>
+        <v>0.983006275669043</v>
       </c>
       <c r="D13">
         <v>0.976858174028987</v>
       </c>
       <c r="E13">
-        <v>1.4416179829439899</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+        <v>1.44161798294399</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
-        <v>-0.75199845082126104</v>
+        <v>-0.751998450821261</v>
       </c>
       <c r="D14">
-        <v>-0.39598482761536302</v>
+        <v>-0.395984827615363</v>
       </c>
       <c r="E14">
-        <v>-0.29043031142040199</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>-0.290430311420402</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
-        <v>0.40478070501389601</v>
+        <v>0.404780705013896</v>
       </c>
       <c r="D15">
-        <v>0.63962144886654104</v>
+        <v>0.639621448866541</v>
       </c>
       <c r="E15">
-        <v>0.41039596022329999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+        <v>0.4103959602233</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
         <v>-1.41026384750747</v>
@@ -3041,32 +2861,32 @@
         <v>-0.269044364431755</v>
       </c>
       <c r="E16">
-        <v>9.0586658239791298E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+        <v>0.0905866582397913</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
         <v>-0.105709302884452</v>
       </c>
       <c r="D17">
-        <v>-0.25108884778781598</v>
+        <v>-0.251088847787816</v>
       </c>
       <c r="E17">
-        <v>-0.19878651280399501</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+        <v>-0.198786512803995</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
         <v>-1.02661929129623</v>
@@ -3075,98 +2895,95 @@
         <v>-1.26262750699747</v>
       </c>
       <c r="E18">
-        <v>-1.1921015273515501</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+        <v>-1.19210152735155</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
-        <v>1.3177110283620199</v>
+        <v>1.31771102836202</v>
       </c>
       <c r="D19">
-        <v>1.2880472692047999</v>
+        <v>1.2880472692048</v>
       </c>
       <c r="E19">
-        <v>1.5309831587774501</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>1.53098315877745</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
-        <v>0.40820898095417801</v>
+        <v>0.408208980954178</v>
       </c>
       <c r="D20">
-        <v>1.0500276907448201</v>
+        <v>1.05002769074482</v>
       </c>
       <c r="E20">
-        <v>1.4171295501935499</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+        <v>1.41712955019355</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
-        <v>1.4028761460241701</v>
+        <v>1.40287614602417</v>
       </c>
       <c r="D21">
-        <v>1.2314519660749701</v>
+        <v>1.23145196607497</v>
       </c>
       <c r="E21">
         <v>1.50806209670647</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
-        <v>-0.66486605652808095</v>
+        <v>-0.664866056528081</v>
       </c>
       <c r="D22">
-        <v>-0.51022603008343204</v>
+        <v>-0.510226030083432</v>
       </c>
       <c r="E22">
-        <v>-0.72124064515279496</v>
+        <v>-0.721240645152795</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
       </c>
       <c r="C1">
         <v>0</v>
@@ -3190,12 +3007,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -3204,7 +3021,7 @@
         <v>-1.5246945056957917</v>
       </c>
       <c r="E2">
-        <v>-1.6117559524070519</v>
+        <v>-1.611755952407052</v>
       </c>
       <c r="F2">
         <v>-1.6146217377845002</v>
@@ -3219,47 +3036,47 @@
         <v>-1.6147478480366781</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>-9.5457785710995141E-2</v>
+        <v>-0.09545778571099514</v>
       </c>
       <c r="E3">
-        <v>-5.3903109597097647E-2</v>
+        <v>-0.05390310959709765</v>
       </c>
       <c r="F3">
-        <v>-2.1542739837201334E-2</v>
+        <v>-0.021542739837201334</v>
       </c>
       <c r="G3">
-        <v>-3.4497691141535431E-3</v>
+        <v>-0.003449769114153543</v>
       </c>
       <c r="H3">
-        <v>5.0533712065816694E-3</v>
+        <v>0.005053371206581669</v>
       </c>
       <c r="I3">
-        <v>7.4319440477687015E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>0.0074319440477687015</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0.11351590063217221</v>
+        <v>0.1135159006321722</v>
       </c>
       <c r="E4">
         <v>0.19525717392912556</v>
@@ -3268,21 +3085,21 @@
         <v>0.25333431182071786</v>
       </c>
       <c r="G4">
-        <v>0.29417887789389841</v>
+        <v>0.2941788778938984</v>
       </c>
       <c r="H4">
         <v>0.32262998579496305</v>
       </c>
       <c r="I4">
-        <v>0.34224551332283282</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>0.3422455133228328</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -3291,7 +3108,7 @@
         <v>0.5909563092708654</v>
       </c>
       <c r="E5">
-        <v>0.91991726606390922</v>
+        <v>0.9199172660639092</v>
       </c>
       <c r="F5">
         <v>1.1282669708449742</v>
@@ -3303,15 +3120,15 @@
         <v>1.3677285223203857</v>
       </c>
       <c r="I5">
-        <v>1.4386667878320649</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+        <v>1.438666787832065</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -3320,65 +3137,65 @@
         <v>-0.29447688973001973</v>
       </c>
       <c r="E6">
-        <v>-0.53465781325293094</v>
+        <v>-0.5346578132529309</v>
       </c>
       <c r="F6">
-        <v>-0.70874526974819196</v>
+        <v>-0.708745269748192</v>
       </c>
       <c r="G6">
-        <v>-0.81462260527027586</v>
+        <v>-0.8146226052702759</v>
       </c>
       <c r="H6">
-        <v>-0.86054006534866079</v>
+        <v>-0.8605400653486608</v>
       </c>
       <c r="I6">
-        <v>-0.86115985356668601</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+        <v>-0.861159853566686</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>7.6338931463816539E-2</v>
+        <v>0.07633893146381654</v>
       </c>
       <c r="E7">
         <v>0.17234228041364585</v>
       </c>
       <c r="F7">
-        <v>0.27392835399743221</v>
+        <v>0.2739283539974322</v>
       </c>
       <c r="G7">
-        <v>0.37204075475130272</v>
+        <v>0.3720407547513027</v>
       </c>
       <c r="H7">
-        <v>0.46171333742927412</v>
+        <v>0.4617133374292741</v>
       </c>
       <c r="I7">
-        <v>0.54075932766897139</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+        <v>0.5407593276689714</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>-4.0012149598054603E-2</v>
+        <v>-0.0400121495980546</v>
       </c>
       <c r="E8">
-        <v>-7.312012605499979E-2</v>
+        <v>-0.07312012605499979</v>
       </c>
       <c r="F8">
         <v>-0.10101576615636461</v>
@@ -3387,18 +3204,18 @@
         <v>-0.12503065869988264</v>
       </c>
       <c r="H8">
-        <v>-0.14616975843375091</v>
+        <v>-0.1461697584337509</v>
       </c>
       <c r="I8">
         <v>-0.16516560358472784</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -3407,27 +3224,27 @@
         <v>0.24283586752823272</v>
       </c>
       <c r="E9">
-        <v>0.40381818464456698</v>
+        <v>0.403818184644567</v>
       </c>
       <c r="F9">
-        <v>0.51545825730735495</v>
+        <v>0.515458257307355</v>
       </c>
       <c r="G9">
-        <v>0.59508226913525053</v>
+        <v>0.5950822691352505</v>
       </c>
       <c r="H9">
-        <v>0.65293663072357111</v>
+        <v>0.6529366307235711</v>
       </c>
       <c r="I9">
-        <v>0.69551525100246758</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+        <v>0.6955152510024676</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -3436,27 +3253,27 @@
         <v>-0.30797521913255055</v>
       </c>
       <c r="E10">
-        <v>-0.56651035779283299</v>
+        <v>-0.566510357792833</v>
       </c>
       <c r="F10">
-        <v>-0.76471137200818429</v>
+        <v>-0.7647113720081843</v>
       </c>
       <c r="G10">
-        <v>-0.89805694376302192</v>
+        <v>-0.8980569437630219</v>
       </c>
       <c r="H10">
-        <v>-0.97015514922408119</v>
+        <v>-0.9701551492240812</v>
       </c>
       <c r="I10">
-        <v>-0.99127220112166003</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+        <v>-0.99127220112166</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -3468,62 +3285,62 @@
         <v>0.47547474734153783</v>
       </c>
       <c r="F11">
-        <v>0.53358452362432063</v>
+        <v>0.5335845236243206</v>
       </c>
       <c r="G11">
-        <v>0.55176088733426121</v>
+        <v>0.5517608873342612</v>
       </c>
       <c r="H11">
         <v>0.5479273878623534</v>
       </c>
       <c r="I11">
-        <v>0.53119309511533919</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+        <v>0.5311930951153392</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
       <c r="D12">
-        <v>-0.18287031437523801</v>
+        <v>-0.182870314375238</v>
       </c>
       <c r="E12">
         <v>-0.27607406995092715</v>
       </c>
       <c r="F12">
-        <v>-0.32134878372788372</v>
+        <v>-0.3213487837278837</v>
       </c>
       <c r="G12">
         <v>-0.34279940634999545</v>
       </c>
       <c r="H12">
-        <v>-0.35283838957866331</v>
+        <v>-0.3528383895786633</v>
       </c>
       <c r="I12">
-        <v>-0.35750972281162918</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+        <v>-0.3575097228116292</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>0.61711808017769876</v>
+        <v>0.6171180801776988</v>
       </c>
       <c r="E13">
-        <v>0.95492981894858431</v>
+        <v>0.9549298189485843</v>
       </c>
       <c r="F13">
         <v>1.1678633317798703</v>
@@ -3538,12 +3355,12 @@
         <v>1.4839515989201006</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -3552,27 +3369,27 @@
         <v>-0.44158522314750914</v>
       </c>
       <c r="E14">
-        <v>-0.59523961112932089</v>
+        <v>-0.5952396111293209</v>
       </c>
       <c r="F14">
-        <v>-0.56755556061912626</v>
+        <v>-0.5675555606191263</v>
       </c>
       <c r="G14">
         <v>-0.46797155253460027</v>
       </c>
       <c r="H14">
-        <v>-0.35640227900986299</v>
+        <v>-0.356402279009863</v>
       </c>
       <c r="I14">
-        <v>-0.25606122082122978</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>-0.2560612208212298</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -3587,21 +3404,21 @@
         <v>0.49092708649979244</v>
       </c>
       <c r="G15">
-        <v>0.53412926419430473</v>
+        <v>0.5341292641943047</v>
       </c>
       <c r="H15">
-        <v>0.55951833461327394</v>
+        <v>0.5595183346132739</v>
       </c>
       <c r="I15">
-        <v>0.57524958718309771</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+        <v>0.5752495871830977</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -3622,15 +3439,15 @@
         <v>-0.23385237005326318</v>
       </c>
       <c r="I16">
-        <v>-0.20391093926790749</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+        <v>-0.2039109392679075</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -3639,27 +3456,27 @@
         <v>-0.10746774774541429</v>
       </c>
       <c r="E17">
-        <v>-0.16898484161814439</v>
+        <v>-0.1689848416181444</v>
       </c>
       <c r="F17">
         <v>-0.20257565349713572</v>
       </c>
       <c r="G17">
-        <v>-0.22016535527150599</v>
+        <v>-0.220165355271506</v>
       </c>
       <c r="H17">
-        <v>-0.22892806290771961</v>
+        <v>-0.2289280629077196</v>
       </c>
       <c r="I17">
         <v>-0.2329747517241616</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -3671,33 +3488,33 @@
         <v>-0.38461538477986873</v>
       </c>
       <c r="F18">
-        <v>-0.57692307730504067</v>
+        <v>-0.5769230773050407</v>
       </c>
       <c r="G18">
-        <v>-0.76923077163692855</v>
+        <v>-0.7692307716369285</v>
       </c>
       <c r="H18">
-        <v>-0.96153846213104999</v>
+        <v>-0.96153846213105</v>
       </c>
       <c r="I18">
         <v>-1.1538461531171527</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>0.75443620081213258</v>
+        <v>0.7544362008121326</v>
       </c>
       <c r="E19">
-        <v>1.1258787366550871</v>
+        <v>1.125878736655087</v>
       </c>
       <c r="F19">
         <v>1.3519718564744132</v>
@@ -3712,12 +3529,12 @@
         <v>1.7090834292782853</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -3726,7 +3543,7 @@
         <v>0.48772456504334705</v>
       </c>
       <c r="E20">
-        <v>0.80007353053327701</v>
+        <v>0.800073530533277</v>
       </c>
       <c r="F20">
         <v>1.0050977451965695</v>
@@ -3741,21 +3558,21 @@
         <v>1.2936133702251116</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>0.90325756799397305</v>
+        <v>0.903257567993973</v>
       </c>
       <c r="E21">
-        <v>1.2554241604617951</v>
+        <v>1.255424160461795</v>
       </c>
       <c r="F21">
         <v>1.4232858173210396</v>
@@ -3770,12 +3587,12 @@
         <v>1.5494617093936773</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -3784,553 +3601,544 @@
         <v>-0.29195874607095557</v>
       </c>
       <c r="E22">
-        <v>-0.50281652156818191</v>
+        <v>-0.5028165215681819</v>
       </c>
       <c r="F22">
         <v>-0.6350304865706865</v>
       </c>
       <c r="G22">
-        <v>-0.70239612104391114</v>
+        <v>-0.7023961210439111</v>
       </c>
       <c r="H22">
-        <v>-0.72371444268079044</v>
+        <v>-0.7237144426807904</v>
       </c>
       <c r="I22">
-        <v>-0.71665760628467101</v>
+        <v>-0.716657606284671</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>DegradationRate</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
         <v>0.34657359027997264</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
         <v>0.23104906018664842</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
-        <v>3.0136833937388925E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>0.030136833937388925</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
-        <v>2.7179999999999999E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+        <v>0.02718</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
-        <v>2.5672117798516494E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+        <v>0.025672117798516494</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
-        <v>1.7328679513998631E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+        <v>0.01732867951399863</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
-        <v>1.1002336199364211E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+        <v>0.01100233619936421</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
-        <v>2.7179999999999999E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+        <v>0.02718</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
-        <v>2.7179999999999999E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+        <v>0.02718</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
-        <v>7.453195489891885E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+        <v>0.007453195489891885</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
-        <v>7.7016353395549478E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+        <v>0.07701635339554948</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
-        <v>2.7179999999999999E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+        <v>0.02718</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
-        <v>6.9314718055994526E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>0.06931471805599453</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
-        <v>4.9510512897138946E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+        <v>0.049510512897138946</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
-        <v>1.6503504299046318E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+        <v>0.016503504299046318</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
-        <v>5.7762265046662105E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+        <v>0.057762265046662105</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
-        <v>1.332975347230664E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+        <v>0.01332975347230664</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
-        <v>1.2602676010180823E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>0.012602676010180823</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
-        <v>3.0136833937388925E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+        <v>0.030136833937388925</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
-        <v>3.0136833937388925E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+        <v>0.030136833937388925</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
-        <v>3.3007008598092635E-2</v>
+        <v>0.033007008598092635</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SystematicName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>StandardName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>production_rates</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>YKL112W</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="C2">
         <v>0.22632780820666573</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>YLR131C</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="C3">
-        <v>0.55521379565059015</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>0.5552137956505901</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>YGL071W</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="C4">
         <v>0.17287454603478603</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>YOR028C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="C5">
         <v>0.16999125421489655</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YPL177C</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="C6">
         <v>0.19433009682781108</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YPR104C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="C7">
         <v>0.22428001203533895</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YGL181W</v>
+      </c>
+      <c r="B8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="C8">
-        <v>5.4375125371813889E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+        <v>0.05437512537181389</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>YOL089C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="C9">
-        <v>9.6231248933555655E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
+        <v>0.09623124893355565</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>YGL073W</v>
+      </c>
+      <c r="B10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="C10">
         <v>0.3658670195100438</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>YMR021C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="C11">
         <v>0.40082067594014675</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>YOL116W</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="C12">
         <v>0.11988807110995572</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>YKL062W</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="C13">
         <v>0.19553557227531512</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>YDR043C</v>
+      </c>
+      <c r="B14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="C14">
-        <v>0.42149594724160672</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
+        <v>0.4214959472416067</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>YKL043W</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="C15">
         <v>0.25140887760964525</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>YNL216W</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="C16">
         <v>0.4695684366567594</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>YBR049C</v>
+      </c>
+      <c r="B17" t="str">
+        <v>REB1</v>
       </c>
       <c r="C17">
         <v>0.10912048970276542</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>YPR065W</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ROX1</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>YER169W</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RPH1</v>
       </c>
       <c r="C19">
-        <v>0.74928855080194068</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>0.7492885508019407</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>YHR206W</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SKN7</v>
       </c>
       <c r="C20">
-        <v>0.71642133761327131</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
+        <v>0.7164213376132713</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>YML007W</v>
+      </c>
+      <c r="B21" t="str">
+        <v>YAP1</v>
       </c>
       <c r="C21">
-        <v>1.1097370215502349</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
+        <v>1.109737021550235</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>YDR259C</v>
+      </c>
+      <c r="B22" t="str">
+        <v>YAP6</v>
       </c>
       <c r="C22">
-        <v>0.17519799830948399</v>
+        <v>0.175197998309484</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>46</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>time</v>
       </c>
       <c r="B1">
         <v>15</v>
@@ -4344,72 +4152,69 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>cols regulators/rows targets</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ABF1</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ACE2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>AFT1</v>
+      </c>
+      <c r="E1" t="str">
+        <v>CIN5</v>
+      </c>
+      <c r="F1" t="str">
+        <v>CUP9</v>
+      </c>
+      <c r="G1" t="str">
+        <v>FHL1</v>
+      </c>
+      <c r="H1" t="str">
+        <v>GTS1</v>
+      </c>
+      <c r="I1" t="str">
+        <v>HAL9</v>
+      </c>
+      <c r="J1" t="str">
+        <v>HSF1</v>
+      </c>
+      <c r="K1" t="str">
+        <v>MAC1</v>
+      </c>
+      <c r="L1" t="str">
+        <v>MSN1</v>
+      </c>
+      <c r="M1" t="str">
+        <v>MSN4</v>
+      </c>
+      <c r="N1" t="str">
+        <v>NRG1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>PHD1</v>
+      </c>
+      <c r="P1" t="str">
+        <v>RAP1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ABF1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -4457,9 +4262,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ACE2</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4507,9 +4312,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AFT1</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -4557,9 +4362,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CIN5</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4607,9 +4412,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CUP9</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4657,9 +4462,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>FHL1</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -4707,9 +4512,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="1" t="s">
-        <v>15</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>GTS1</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -4757,9 +4562,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
-      <c r="A9" s="1" t="s">
-        <v>17</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>HAL9</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -4807,9 +4612,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
-      <c r="A10" s="1" t="s">
-        <v>19</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>HSF1</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -4857,9 +4662,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
-      <c r="A11" s="1" t="s">
-        <v>21</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>MAC1</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -4907,9 +4712,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
-      <c r="A12" s="1" t="s">
-        <v>23</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>MSN1</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -4957,9 +4762,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
-      <c r="A13" s="1" t="s">
-        <v>25</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>MSN4</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -5007,9 +4812,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
-      <c r="A14" s="1" t="s">
-        <v>27</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NRG1</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -5057,9 +4862,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
-      <c r="A15" s="1" t="s">
-        <v>29</v>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PHD1</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -5107,9 +4912,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="1" t="s">
-        <v>31</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>RAP1</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -5158,12 +4963,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:P16"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>